<commit_message>
data is collected again with gemini + additional genre, feature ext is done, classifier is going to be built
</commit_message>
<xml_diff>
--- a/data/prompts.xlsx
+++ b/data/prompts.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erdem\Desktop\nlp_project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E310CE3-1B7C-45BF-83B4-335E98FB6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF1FCB67-2239-4317-81E4-CA4DB98527FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="2928" windowWidth="17280" windowHeight="8976" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="129">
   <si>
     <t>category</t>
   </si>
@@ -192,13 +203,226 @@
     <t>What do you think of manager who constantly monitors and controls every detail of their team's work? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
   </si>
   <si>
-    <t>What do you think is the best way to deal with a disagreement between close friends? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
-  </si>
-  <si>
     <t>What do you think is the role of luck in a person's life outcomes? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
   </si>
   <si>
     <t>What do you think is the most important quality in a romantic partner? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>dialogue</t>
+  </si>
+  <si>
+    <t>Describe a conversation between two old friends who meet after years apart and discuss how their lives have changed. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two siblings said to each other when one of them decided to move abroad permanently. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between a student and a professor after the student received an unexpectedly low grade. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two colleagues said to each other when they disagreed about an important work decision. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between a parent and an adult child who has just announced a major life decision the parent disapproves of. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two strangers said to each other after being stuck together in a delayed train for several hours. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between two friends where one admits they have been struggling silently for a long time. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what a job candidate and an interviewer said to each other during an unexpectedly honest interview. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between two neighbors who have never spoken before but finally meet during a power outage. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two friends said to each other the night before one of them left for a new life in another country. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between a doctor and a patient who has just received life-changing news and is trying to process it calmly. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two former romantic partners said to each other when they unexpectedly ran into each other years after their breakup. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between a mentor and a young professional who is about to make a decision that could define their career. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two teammates said to each other after losing an important competition they had worked months to prepare for. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between a traveler and a local resident who gives them unexpected advice that changes how they see the place they are visiting. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between two researchers who strongly disagree about the direction of their shared project. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what two friends said to each other when one of them admitted they had made a serious mistake that affected the other. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe a conversation between an elderly person and a young stranger who sit next to each other on a long flight. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what a person said to their closest friend on the night they both realized their friendship had quietly grown apart over the years. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Describe what a teacher said to a student who had given up on themselves, and how the student responded. Write it as a narrative account of the dialogue, not as a script. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why some languages are considered harder to learn than others. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why people who grow up bilingual tend to think differently than those who speak only one language. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why cities tend to be significantly warmer than the surrounding countryside. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why deep-sea creatures often look so different from land and shallow-water animals. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why childhood memories are often more vivid than memories from last week. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain how the human brain forms and stores long-term memories. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why some materials conduct electricity while others do not. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain how earthquakes occur and why some regions are more prone to them. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain why procrastination is so common even when people know it causes them stress. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Explain how black holes form and why nothing can escape their gravity. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>What do you think makes a good morning? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a house feel like a home? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a good book? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a good teacher? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a conversation truly memorable? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a piece of music stay in your head long after you have heard it? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a foreign language sound beautiful to someone who does not speak it? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a rainy day feel cozy rather than gloomy? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes some daily routines feel meaningful rather than mechanical? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes an apology feel sincere? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>What do you think makes a weekend feel truly restful rather than just empty? Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Share your personal opinion. You do not need to argue or prove a point, just express what you think and why.</t>
+  </si>
+  <si>
+    <t>Compare traveling alone and traveling with friends in terms of experience and personal growth. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare how introverts and extroverts tend to handle social conflict differently. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare the social dynamics of online friendships and in-person friendships. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare how people experience time differently when they are busy versus when they are bored. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare the way children and adults approach learning a new skill. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare the mental effects of regular exercise and meditation as stress management strategies. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare how the same historical event is often remembered differently by the two sides involved. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare the experience of failing publicly and failing privately in terms of psychological impact. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare short-term and long-term thinking in personal financial decisions. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Compare the experience of living alone and living with roommates in terms of daily life and personal development. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the last hour before a university student submits their thesis after months of work. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the moment a young adult returns to their childhood home after years of living abroad. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the final moments of a small family-owned bookstore on its last day before permanently closing. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the experience of a person who wakes up in an unfamiliar place with no memory of how they got there. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the moment a person opens a letter they have been too afraid to read for weeks. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the experience of a person sitting alone in a café waiting for someone who is very late. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the events of a person's last day at a job they have held for ten years. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the moment a person realizes mid-conversation that they have been completely misunderstood. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the experience of a person who gets lost in a forest and must find their way back before dark. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Narrate the events that unfold when a person misses their flight and has to spend the night at the airport. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points.</t>
+  </si>
+  <si>
+    <t>Argue whether people who pursue comfort throughout their lives ultimately lead less meaningful existences. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether the pressure to be productive has become a form of social control in modern society. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether humans are naturally more inclined toward cooperation than competition. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether the way a society treats its elderly reveals its true values. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether most people choose comfort over genuine personal growth when given the choice. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether privacy is becoming an outdated concept in the digital age. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether it is possible to be truly objective when forming political opinions. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether technology has made people more impatient in ways that harm their relationships. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether success achieved through luck deserves the same respect as success achieved through effort. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
+  </si>
+  <si>
+    <t>Argue whether a person's cultural background should influence how they are judged in a professional setting. Answer in English. Write approximately 150 words. Write in paragraph form, not bullet points. Take a clear stance and defend it. Do not present both sides equally.</t>
   </si>
 </sst>
 </file>
@@ -516,7 +740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
@@ -648,10 +872,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -659,10 +883,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -670,10 +894,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -681,10 +905,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -692,10 +916,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -703,10 +927,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -714,10 +938,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -725,10 +949,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -736,10 +960,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>56</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -747,10 +971,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -758,10 +982,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -769,10 +993,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -780,10 +1004,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -791,10 +1015,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C25" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -802,10 +1026,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -813,10 +1037,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -824,10 +1048,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -835,10 +1059,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -846,10 +1070,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -857,10 +1081,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -868,10 +1092,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -879,10 +1103,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C33" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -890,10 +1114,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C34" t="s">
-        <v>20</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -901,10 +1125,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C35" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -912,10 +1136,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C36" t="s">
-        <v>22</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -923,10 +1147,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C37" t="s">
-        <v>23</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -934,10 +1158,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -945,10 +1169,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C39" t="s">
-        <v>25</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -956,10 +1180,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C40" t="s">
-        <v>26</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -967,10 +1191,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s">
-        <v>27</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -978,10 +1202,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C42" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -989,10 +1213,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -1000,10 +1224,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -1011,10 +1235,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C45" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -1022,10 +1246,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -1033,10 +1257,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C47" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -1044,10 +1268,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C48" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -1055,10 +1279,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C49" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -1066,10 +1290,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -1077,10 +1301,780 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>6</v>
+      </c>
+      <c r="C53" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>6</v>
+      </c>
+      <c r="C55" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
         <v>5</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C82" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>5</v>
+      </c>
+      <c r="C83" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>5</v>
+      </c>
+      <c r="C84" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>5</v>
+      </c>
+      <c r="C85" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>5</v>
+      </c>
+      <c r="C86" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>5</v>
+      </c>
+      <c r="C93" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>5</v>
+      </c>
+      <c r="C94" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>5</v>
+      </c>
+      <c r="C95" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>5</v>
+      </c>
+      <c r="C96" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>5</v>
+      </c>
+      <c r="C97" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>5</v>
+      </c>
+      <c r="C98" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>5</v>
+      </c>
+      <c r="C99" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C100" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>5</v>
+      </c>
+      <c r="C101" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>57</v>
+      </c>
+      <c r="C102" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>57</v>
+      </c>
+      <c r="C103" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>57</v>
+      </c>
+      <c r="C104" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>57</v>
+      </c>
+      <c r="C105" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>57</v>
+      </c>
+      <c r="C106" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>57</v>
+      </c>
+      <c r="C107" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>57</v>
+      </c>
+      <c r="C108" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>57</v>
+      </c>
+      <c r="C109" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>57</v>
+      </c>
+      <c r="C110" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>57</v>
+      </c>
+      <c r="C111" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>57</v>
+      </c>
+      <c r="C112" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>57</v>
+      </c>
+      <c r="C113" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="s">
+        <v>57</v>
+      </c>
+      <c r="C114" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>57</v>
+      </c>
+      <c r="C115" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>57</v>
+      </c>
+      <c r="C116" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>57</v>
+      </c>
+      <c r="C117" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>57</v>
+      </c>
+      <c r="C118" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>57</v>
+      </c>
+      <c r="C119" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>57</v>
+      </c>
+      <c r="C120" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>57</v>
+      </c>
+      <c r="C121" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>